<commit_message>
Version 1.2.0.0 Public Beta
</commit_message>
<xml_diff>
--- a/MapLab3D_ProjectParameters_1_2_0_0_Colors_Database.xlsx
+++ b/MapLab3D_ProjectParameters_1_2_0_0_Colors_Database.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Daten\Projekte\MapLab3D\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{79DB998E-42CD-456A-BF25-EA0B6E91C8A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4DBFD96F-E1CE-4384-9AE2-395511867D4E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-105" yWindow="210" windowWidth="24180" windowHeight="14595" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4680" yWindow="4680" windowWidth="34425" windowHeight="13275" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7660" uniqueCount="332">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="7898" uniqueCount="343">
   <si>
     <t>N</t>
   </si>
@@ -1040,6 +1040,39 @@
   <si>
     <t>RAL 5013</t>
   </si>
+  <si>
+    <t>Pearl Night Blue</t>
+  </si>
+  <si>
+    <t>RAL 5026</t>
+  </si>
+  <si>
+    <t>https://shop.fillamentum.com/collections/pla-extrafill-filament/products/pla-extrafill-pearl-night-blue-1kg</t>
+  </si>
+  <si>
+    <t>PrimaValue PLA+</t>
+  </si>
+  <si>
+    <t>PrimaCreator</t>
+  </si>
+  <si>
+    <t>https://primacreator.com/collections/filament-pla/products/primavalue-pla?variant=48794154828123</t>
+  </si>
+  <si>
+    <t>https://primacreator.com/collections/filament-pla/products/primavalue-pla?variant=48794154926427</t>
+  </si>
+  <si>
+    <t>White</t>
+  </si>
+  <si>
+    <t>Matt Polar Blue</t>
+  </si>
+  <si>
+    <t>https://www.formfutura.com/filaments/pla/easyfil-epla</t>
+  </si>
+  <si>
+    <t>PLAE-175MTPB-01000</t>
+  </si>
 </sst>
 </file>
 
@@ -1115,7 +1148,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="83">
+  <fills count="85">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1608,6 +1641,18 @@
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FF323478"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFD7F6FE"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
   </fills>
   <borders count="20">
     <border>
@@ -1831,7 +1876,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="239">
+  <cellXfs count="245">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="49" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
@@ -2534,6 +2579,24 @@
     <xf numFmtId="0" fontId="9" fillId="45" borderId="11" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="83" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="83" borderId="11" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="73" borderId="11" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="7" borderId="11" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="84" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="84" borderId="11" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="8" fillId="77" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
@@ -2552,6 +2615,7 @@
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFD7F6FE"/>
       <color rgb="FFC8307B"/>
       <color rgb="FF926AA6"/>
       <color rgb="FFAEAEAE"/>
@@ -2561,7 +2625,6 @@
       <color rgb="FF000000"/>
       <color rgb="FF191919"/>
       <color rgb="FF6E6661"/>
-      <color rgb="FF4E3630"/>
     </mruColors>
   </colors>
   <extLst>
@@ -2838,7 +2901,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:R1295"/>
+  <dimension ref="A1:R1334"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="12.75" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="5.140625" style="11" bestFit="1" customWidth="1"/>
@@ -2860,70 +2923,70 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="18" x14ac:dyDescent="0.25">
-      <c r="A1" s="236" t="s">
+      <c r="A1" s="242" t="s">
         <v>325</v>
       </c>
-      <c r="B1" s="237"/>
-      <c r="C1" s="237"/>
-      <c r="D1" s="237"/>
-      <c r="E1" s="237"/>
-      <c r="F1" s="237"/>
-      <c r="G1" s="237"/>
-      <c r="H1" s="237"/>
-      <c r="I1" s="237"/>
-      <c r="J1" s="237"/>
-      <c r="K1" s="237"/>
-      <c r="L1" s="237"/>
-      <c r="M1" s="237"/>
-      <c r="N1" s="237"/>
-      <c r="O1" s="237"/>
-      <c r="P1" s="237"/>
-      <c r="Q1" s="237"/>
-      <c r="R1" s="238"/>
+      <c r="B1" s="243"/>
+      <c r="C1" s="243"/>
+      <c r="D1" s="243"/>
+      <c r="E1" s="243"/>
+      <c r="F1" s="243"/>
+      <c r="G1" s="243"/>
+      <c r="H1" s="243"/>
+      <c r="I1" s="243"/>
+      <c r="J1" s="243"/>
+      <c r="K1" s="243"/>
+      <c r="L1" s="243"/>
+      <c r="M1" s="243"/>
+      <c r="N1" s="243"/>
+      <c r="O1" s="243"/>
+      <c r="P1" s="243"/>
+      <c r="Q1" s="243"/>
+      <c r="R1" s="244"/>
     </row>
     <row r="2" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="236" t="s">
+      <c r="A2" s="242" t="s">
         <v>328</v>
       </c>
-      <c r="B2" s="237"/>
-      <c r="C2" s="237"/>
-      <c r="D2" s="237"/>
-      <c r="E2" s="237"/>
-      <c r="F2" s="237"/>
-      <c r="G2" s="237"/>
-      <c r="H2" s="237"/>
-      <c r="I2" s="237"/>
-      <c r="J2" s="237"/>
-      <c r="K2" s="237"/>
-      <c r="L2" s="237"/>
-      <c r="M2" s="237"/>
-      <c r="N2" s="237"/>
-      <c r="O2" s="237"/>
-      <c r="P2" s="237"/>
-      <c r="Q2" s="237"/>
-      <c r="R2" s="238"/>
+      <c r="B2" s="243"/>
+      <c r="C2" s="243"/>
+      <c r="D2" s="243"/>
+      <c r="E2" s="243"/>
+      <c r="F2" s="243"/>
+      <c r="G2" s="243"/>
+      <c r="H2" s="243"/>
+      <c r="I2" s="243"/>
+      <c r="J2" s="243"/>
+      <c r="K2" s="243"/>
+      <c r="L2" s="243"/>
+      <c r="M2" s="243"/>
+      <c r="N2" s="243"/>
+      <c r="O2" s="243"/>
+      <c r="P2" s="243"/>
+      <c r="Q2" s="243"/>
+      <c r="R2" s="244"/>
     </row>
     <row r="3" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A3" s="236" t="s">
+      <c r="A3" s="242" t="s">
         <v>326</v>
       </c>
-      <c r="B3" s="237"/>
-      <c r="C3" s="237"/>
-      <c r="D3" s="237"/>
-      <c r="E3" s="237"/>
-      <c r="F3" s="237"/>
-      <c r="G3" s="237"/>
-      <c r="H3" s="237"/>
-      <c r="I3" s="237"/>
-      <c r="J3" s="237"/>
-      <c r="K3" s="237"/>
-      <c r="L3" s="237"/>
-      <c r="M3" s="237"/>
-      <c r="N3" s="237"/>
-      <c r="O3" s="237"/>
-      <c r="P3" s="237"/>
-      <c r="Q3" s="237"/>
-      <c r="R3" s="238"/>
+      <c r="B3" s="243"/>
+      <c r="C3" s="243"/>
+      <c r="D3" s="243"/>
+      <c r="E3" s="243"/>
+      <c r="F3" s="243"/>
+      <c r="G3" s="243"/>
+      <c r="H3" s="243"/>
+      <c r="I3" s="243"/>
+      <c r="J3" s="243"/>
+      <c r="K3" s="243"/>
+      <c r="L3" s="243"/>
+      <c r="M3" s="243"/>
+      <c r="N3" s="243"/>
+      <c r="O3" s="243"/>
+      <c r="P3" s="243"/>
+      <c r="Q3" s="243"/>
+      <c r="R3" s="244"/>
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" s="14" t="s">
@@ -3075,7 +3138,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A8" s="7" t="s">
         <v>2</v>
       </c>
@@ -3579,7 +3642,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="21" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A21" s="7" t="s">
         <v>2</v>
       </c>
@@ -4083,7 +4146,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="34" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A34" s="7" t="s">
         <v>2</v>
       </c>
@@ -4585,7 +4648,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="47" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="47" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A47" s="7" t="s">
         <v>2</v>
       </c>
@@ -5089,7 +5152,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="60" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A60" s="7" t="s">
         <v>2</v>
       </c>
@@ -5593,7 +5656,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="73" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A73" s="7" t="s">
         <v>2</v>
       </c>
@@ -6097,7 +6160,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="86" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="86" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A86" s="7" t="s">
         <v>2</v>
       </c>
@@ -6601,7 +6664,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="99" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="99" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A99" s="7" t="s">
         <v>2</v>
       </c>
@@ -7105,7 +7168,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="112" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="112" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A112" s="7" t="s">
         <v>2</v>
       </c>
@@ -7605,7 +7668,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="125" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="125" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A125" s="7" t="s">
         <v>2</v>
       </c>
@@ -8111,7 +8174,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="138" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="138" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A138" s="7" t="s">
         <v>2</v>
       </c>
@@ -8617,7 +8680,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="151" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A151" s="7" t="s">
         <v>2</v>
       </c>
@@ -9121,7 +9184,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="164" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="164" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A164" s="7" t="s">
         <v>2</v>
       </c>
@@ -9625,7 +9688,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="177" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="177" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A177" s="7" t="s">
         <v>2</v>
       </c>
@@ -10127,7 +10190,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="190" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="190" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A190" s="7" t="s">
         <v>2</v>
       </c>
@@ -10625,7 +10688,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="203" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="203" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A203" s="7" t="s">
         <v>2</v>
       </c>
@@ -11129,7 +11192,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="216" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="216" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A216" s="7" t="s">
         <v>2</v>
       </c>
@@ -11633,7 +11696,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="229" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="229" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A229" s="7" t="s">
         <v>2</v>
       </c>
@@ -12137,7 +12200,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="242" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="242" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A242" s="7" t="s">
         <v>2</v>
       </c>
@@ -12641,7 +12704,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="255" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="255" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A255" s="7" t="s">
         <v>2</v>
       </c>
@@ -13145,7 +13208,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="268" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="268" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A268" s="7" t="s">
         <v>2</v>
       </c>
@@ -13649,7 +13712,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="281" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="281" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A281" s="7" t="s">
         <v>2</v>
       </c>
@@ -14151,7 +14214,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="294" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="294" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A294" s="7" t="s">
         <v>2</v>
       </c>
@@ -14643,7 +14706,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="307" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="307" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A307" s="7" t="s">
         <v>2</v>
       </c>
@@ -15135,7 +15198,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="320" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="320" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A320" s="7" t="s">
         <v>2</v>
       </c>
@@ -15627,7 +15690,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="333" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="333" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A333" s="7" t="s">
         <v>2</v>
       </c>
@@ -16119,7 +16182,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="346" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="346" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A346" s="7" t="s">
         <v>2</v>
       </c>
@@ -16611,7 +16674,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="359" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="359" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A359" s="7" t="s">
         <v>2</v>
       </c>
@@ -17103,7 +17166,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="372" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="372" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A372" s="7" t="s">
         <v>2</v>
       </c>
@@ -17609,7 +17672,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="385" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="385" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A385" s="7" t="s">
         <v>2</v>
       </c>
@@ -18115,7 +18178,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="398" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="398" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A398" s="7" t="s">
         <v>2</v>
       </c>
@@ -18621,7 +18684,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="411" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="411" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A411" s="7" t="s">
         <v>2</v>
       </c>
@@ -19125,7 +19188,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="424" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="424" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A424" s="7" t="s">
         <v>2</v>
       </c>
@@ -19629,7 +19692,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="437" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="437" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A437" s="7" t="s">
         <v>2</v>
       </c>
@@ -20133,7 +20196,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="450" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="450" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A450" s="7" t="s">
         <v>2</v>
       </c>
@@ -20639,7 +20702,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="463" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="463" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A463" s="7" t="s">
         <v>2</v>
       </c>
@@ -21143,7 +21206,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="476" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="476" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A476" s="7" t="s">
         <v>2</v>
       </c>
@@ -21647,7 +21710,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="489" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="489" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A489" s="7" t="s">
         <v>2</v>
       </c>
@@ -22151,7 +22214,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="502" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="502" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A502" s="7" t="s">
         <v>2</v>
       </c>
@@ -22655,7 +22718,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="515" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="515" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A515" s="7" t="s">
         <v>2</v>
       </c>
@@ -23159,7 +23222,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="528" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="528" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A528" s="7" t="s">
         <v>2</v>
       </c>
@@ -23663,7 +23726,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="541" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="541" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A541" s="7" t="s">
         <v>2</v>
       </c>
@@ -24167,7 +24230,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="554" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="554" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A554" s="7" t="s">
         <v>2</v>
       </c>
@@ -24671,7 +24734,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="567" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="567" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A567" s="7" t="s">
         <v>2</v>
       </c>
@@ -25175,7 +25238,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="580" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="580" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A580" s="7" t="s">
         <v>2</v>
       </c>
@@ -25679,7 +25742,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="593" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="593" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A593" s="7" t="s">
         <v>2</v>
       </c>
@@ -26183,7 +26246,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="606" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="606" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A606" s="7" t="s">
         <v>2</v>
       </c>
@@ -26687,7 +26750,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="619" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="619" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A619" s="7" t="s">
         <v>2</v>
       </c>
@@ -27189,7 +27252,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="632" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="632" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A632" s="7" t="s">
         <v>2</v>
       </c>
@@ -27693,7 +27756,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="645" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="645" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A645" s="7" t="s">
         <v>2</v>
       </c>
@@ -28197,7 +28260,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="658" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="658" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A658" s="7" t="s">
         <v>2</v>
       </c>
@@ -28701,7 +28764,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="671" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="671" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A671" s="7" t="s">
         <v>2</v>
       </c>
@@ -29203,7 +29266,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="684" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="684" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A684" s="7" t="s">
         <v>2</v>
       </c>
@@ -29705,7 +29768,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="697" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="697" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A697" s="7" t="s">
         <v>2</v>
       </c>
@@ -30207,7 +30270,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="710" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="710" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A710" s="7" t="s">
         <v>2</v>
       </c>
@@ -30709,7 +30772,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="723" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="723" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A723" s="7" t="s">
         <v>2</v>
       </c>
@@ -31211,7 +31274,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="736" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="736" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A736" s="7" t="s">
         <v>2</v>
       </c>
@@ -31715,7 +31778,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="749" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="749" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A749" s="7" t="s">
         <v>2</v>
       </c>
@@ -32219,7 +32282,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="762" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="762" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A762" s="7" t="s">
         <v>2</v>
       </c>
@@ -32711,7 +32774,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="775" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="775" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A775" s="7" t="s">
         <v>2</v>
       </c>
@@ -33215,7 +33278,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="788" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="788" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A788" s="7" t="s">
         <v>2</v>
       </c>
@@ -33719,7 +33782,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="801" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="801" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A801" s="7" t="s">
         <v>2</v>
       </c>
@@ -34223,7 +34286,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="814" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="814" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A814" s="7" t="s">
         <v>2</v>
       </c>
@@ -34727,7 +34790,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="827" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="827" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A827" s="7" t="s">
         <v>2</v>
       </c>
@@ -35231,7 +35294,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="840" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="840" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A840" s="7" t="s">
         <v>2</v>
       </c>
@@ -35735,7 +35798,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="853" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="853" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A853" s="7" t="s">
         <v>2</v>
       </c>
@@ -36241,7 +36304,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="866" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="866" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A866" s="7" t="s">
         <v>2</v>
       </c>
@@ -36747,7 +36810,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="879" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="879" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A879" s="7" t="s">
         <v>2</v>
       </c>
@@ -37251,7 +37314,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="892" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="892" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A892" s="7" t="s">
         <v>2</v>
       </c>
@@ -37757,7 +37820,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="905" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="905" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A905" s="7" t="s">
         <v>2</v>
       </c>
@@ -38263,7 +38326,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="918" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="918" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A918" s="7" t="s">
         <v>2</v>
       </c>
@@ -38767,7 +38830,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="931" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="931" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A931" s="7" t="s">
         <v>2</v>
       </c>
@@ -39271,7 +39334,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="944" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="944" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A944" s="7" t="s">
         <v>2</v>
       </c>
@@ -39775,7 +39838,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="957" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="957" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A957" s="7" t="s">
         <v>2</v>
       </c>
@@ -40279,7 +40342,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="970" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="970" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A970" s="7" t="s">
         <v>2</v>
       </c>
@@ -40785,7 +40848,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="983" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="983" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A983" s="7" t="s">
         <v>2</v>
       </c>
@@ -41291,7 +41354,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="996" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="996" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A996" s="7" t="s">
         <v>2</v>
       </c>
@@ -41797,7 +41860,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="1009" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1009" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A1009" s="7" t="s">
         <v>2</v>
       </c>
@@ -42303,7 +42366,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="1022" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1022" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A1022" s="7" t="s">
         <v>2</v>
       </c>
@@ -42809,7 +42872,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="1035" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1035" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A1035" s="7" t="s">
         <v>2</v>
       </c>
@@ -43315,7 +43378,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="1048" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1048" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A1048" s="7" t="s">
         <v>2</v>
       </c>
@@ -43821,7 +43884,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="1061" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1061" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A1061" s="7" t="s">
         <v>2</v>
       </c>
@@ -44327,7 +44390,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="1074" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1074" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A1074" s="7" t="s">
         <v>2</v>
       </c>
@@ -44831,7 +44894,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="1087" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1087" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A1087" s="7" t="s">
         <v>2</v>
       </c>
@@ -45335,7 +45398,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="1100" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1100" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A1100" s="7" t="s">
         <v>2</v>
       </c>
@@ -45839,7 +45902,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="1113" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1113" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A1113" s="7" t="s">
         <v>2</v>
       </c>
@@ -46345,7 +46408,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="1126" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1126" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A1126" s="7" t="s">
         <v>2</v>
       </c>
@@ -46849,7 +46912,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="1139" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1139" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A1139" s="7" t="s">
         <v>2</v>
       </c>
@@ -47355,7 +47418,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="1152" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1152" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A1152" s="7" t="s">
         <v>2</v>
       </c>
@@ -47859,7 +47922,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="1165" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1165" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A1165" s="7" t="s">
         <v>2</v>
       </c>
@@ -48365,7 +48428,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="1178" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1178" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A1178" s="7" t="s">
         <v>2</v>
       </c>
@@ -48869,7 +48932,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="1191" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1191" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A1191" s="7" t="s">
         <v>2</v>
       </c>
@@ -49375,7 +49438,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="1204" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1204" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A1204" s="7" t="s">
         <v>2</v>
       </c>
@@ -49879,7 +49942,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="1217" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1217" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A1217" s="7" t="s">
         <v>2</v>
       </c>
@@ -50374,8 +50437,8 @@
       <c r="L1229" s="30"/>
       <c r="M1229" s="80"/>
       <c r="N1229" s="37"/>
-      <c r="O1229" s="166">
-        <v>249</v>
+      <c r="O1229" s="236">
+        <v>50</v>
       </c>
       <c r="P1229" s="10"/>
       <c r="Q1229" s="43"/>
@@ -50383,7 +50446,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="1230" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1230" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A1230" s="7" t="s">
         <v>2</v>
       </c>
@@ -50415,8 +50478,8 @@
       <c r="L1230" s="30"/>
       <c r="M1230" s="80"/>
       <c r="N1230" s="37"/>
-      <c r="O1230" s="166">
-        <v>249</v>
+      <c r="O1230" s="236">
+        <v>52</v>
       </c>
       <c r="P1230" s="10"/>
       <c r="Q1230" s="43"/>
@@ -50456,8 +50519,8 @@
       <c r="L1231" s="30"/>
       <c r="M1231" s="80"/>
       <c r="N1231" s="37"/>
-      <c r="O1231" s="166">
-        <v>249</v>
+      <c r="O1231" s="236">
+        <v>120</v>
       </c>
       <c r="P1231" s="10"/>
       <c r="Q1231" s="43"/>
@@ -50493,7 +50556,9 @@
       <c r="L1232" s="10"/>
       <c r="M1232" s="40"/>
       <c r="N1232" s="37"/>
-      <c r="O1232" s="166"/>
+      <c r="O1232" s="236" t="s">
+        <v>332</v>
+      </c>
       <c r="P1232" s="10"/>
       <c r="Q1232" s="44" t="s">
         <v>15</v>
@@ -50530,7 +50595,9 @@
       <c r="L1233" s="10"/>
       <c r="M1233" s="40"/>
       <c r="N1233" s="37"/>
-      <c r="O1233" s="166"/>
+      <c r="O1233" s="236" t="s">
+        <v>333</v>
+      </c>
       <c r="P1233" s="10"/>
       <c r="Q1233" s="44" t="s">
         <v>15</v>
@@ -50567,7 +50634,7 @@
       <c r="L1234" s="10"/>
       <c r="M1234" s="40"/>
       <c r="N1234" s="37"/>
-      <c r="O1234" s="166"/>
+      <c r="O1234" s="236"/>
       <c r="P1234" s="10"/>
       <c r="Q1234" s="44" t="s">
         <v>15</v>
@@ -50604,7 +50671,9 @@
       <c r="L1235" s="10"/>
       <c r="M1235" s="40"/>
       <c r="N1235" s="37"/>
-      <c r="O1235" s="166"/>
+      <c r="O1235" s="236" t="s">
+        <v>23</v>
+      </c>
       <c r="P1235" s="10"/>
       <c r="Q1235" s="44" t="s">
         <v>15</v>
@@ -50641,7 +50710,9 @@
       <c r="L1236" s="10"/>
       <c r="M1236" s="40"/>
       <c r="N1236" s="37"/>
-      <c r="O1236" s="166"/>
+      <c r="O1236" s="236" t="s">
+        <v>28</v>
+      </c>
       <c r="P1236" s="10"/>
       <c r="Q1236" s="44" t="s">
         <v>15</v>
@@ -50678,7 +50749,9 @@
       <c r="L1237" s="10"/>
       <c r="M1237" s="40"/>
       <c r="N1237" s="37"/>
-      <c r="O1237" s="166"/>
+      <c r="O1237" s="236" t="s">
+        <v>31</v>
+      </c>
       <c r="P1237" s="10"/>
       <c r="Q1237" s="44" t="s">
         <v>15</v>
@@ -50687,7 +50760,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="1238" spans="1:18" ht="14.25" x14ac:dyDescent="0.25">
+    <row r="1238" spans="1:18" ht="15" x14ac:dyDescent="0.25">
       <c r="A1238" s="46" t="s">
         <v>2</v>
       </c>
@@ -50715,7 +50788,9 @@
       <c r="L1238" s="52"/>
       <c r="M1238" s="54"/>
       <c r="N1238" s="55"/>
-      <c r="O1238" s="167"/>
+      <c r="O1238" s="237" t="s">
+        <v>334</v>
+      </c>
       <c r="P1238" s="52"/>
       <c r="Q1238" s="57" t="s">
         <v>15</v>
@@ -50866,8 +50941,8 @@
       <c r="L1242" s="30"/>
       <c r="M1242" s="80"/>
       <c r="N1242" s="37"/>
-      <c r="O1242" s="166">
-        <v>249</v>
+      <c r="O1242" s="210">
+        <v>25</v>
       </c>
       <c r="P1242" s="10"/>
       <c r="Q1242" s="43"/>
@@ -50875,7 +50950,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="1243" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1243" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A1243" s="7" t="s">
         <v>2</v>
       </c>
@@ -50907,8 +50982,8 @@
       <c r="L1243" s="30"/>
       <c r="M1243" s="80"/>
       <c r="N1243" s="37"/>
-      <c r="O1243" s="166">
-        <v>249</v>
+      <c r="O1243" s="210">
+        <v>25</v>
       </c>
       <c r="P1243" s="10"/>
       <c r="Q1243" s="43"/>
@@ -50948,8 +51023,8 @@
       <c r="L1244" s="30"/>
       <c r="M1244" s="80"/>
       <c r="N1244" s="37"/>
-      <c r="O1244" s="166">
-        <v>249</v>
+      <c r="O1244" s="210">
+        <v>25</v>
       </c>
       <c r="P1244" s="10"/>
       <c r="Q1244" s="43"/>
@@ -50985,7 +51060,9 @@
       <c r="L1245" s="10"/>
       <c r="M1245" s="40"/>
       <c r="N1245" s="37"/>
-      <c r="O1245" s="166"/>
+      <c r="O1245" s="210" t="s">
+        <v>120</v>
+      </c>
       <c r="P1245" s="10"/>
       <c r="Q1245" s="44" t="s">
         <v>15</v>
@@ -51022,7 +51099,7 @@
       <c r="L1246" s="10"/>
       <c r="M1246" s="40"/>
       <c r="N1246" s="37"/>
-      <c r="O1246" s="166"/>
+      <c r="O1246" s="210"/>
       <c r="P1246" s="10"/>
       <c r="Q1246" s="44" t="s">
         <v>15</v>
@@ -51059,7 +51136,7 @@
       <c r="L1247" s="10"/>
       <c r="M1247" s="40"/>
       <c r="N1247" s="37"/>
-      <c r="O1247" s="166"/>
+      <c r="O1247" s="210"/>
       <c r="P1247" s="10"/>
       <c r="Q1247" s="44" t="s">
         <v>15</v>
@@ -51096,7 +51173,9 @@
       <c r="L1248" s="10"/>
       <c r="M1248" s="40"/>
       <c r="N1248" s="37"/>
-      <c r="O1248" s="166"/>
+      <c r="O1248" s="210" t="s">
+        <v>23</v>
+      </c>
       <c r="P1248" s="10"/>
       <c r="Q1248" s="44" t="s">
         <v>15</v>
@@ -51133,7 +51212,9 @@
       <c r="L1249" s="10"/>
       <c r="M1249" s="40"/>
       <c r="N1249" s="37"/>
-      <c r="O1249" s="166"/>
+      <c r="O1249" s="210" t="s">
+        <v>335</v>
+      </c>
       <c r="P1249" s="10"/>
       <c r="Q1249" s="44" t="s">
         <v>15</v>
@@ -51170,7 +51251,9 @@
       <c r="L1250" s="10"/>
       <c r="M1250" s="40"/>
       <c r="N1250" s="37"/>
-      <c r="O1250" s="166"/>
+      <c r="O1250" s="210" t="s">
+        <v>336</v>
+      </c>
       <c r="P1250" s="10"/>
       <c r="Q1250" s="44" t="s">
         <v>15</v>
@@ -51179,7 +51262,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="1251" spans="1:18" ht="14.25" x14ac:dyDescent="0.25">
+    <row r="1251" spans="1:18" ht="15" x14ac:dyDescent="0.25">
       <c r="A1251" s="46" t="s">
         <v>2</v>
       </c>
@@ -51207,7 +51290,9 @@
       <c r="L1251" s="52"/>
       <c r="M1251" s="54"/>
       <c r="N1251" s="55"/>
-      <c r="O1251" s="167"/>
+      <c r="O1251" s="238" t="s">
+        <v>337</v>
+      </c>
       <c r="P1251" s="52"/>
       <c r="Q1251" s="57" t="s">
         <v>15</v>
@@ -51358,8 +51443,8 @@
       <c r="L1255" s="30"/>
       <c r="M1255" s="80"/>
       <c r="N1255" s="37"/>
-      <c r="O1255" s="166">
-        <v>249</v>
+      <c r="O1255" s="218">
+        <v>255</v>
       </c>
       <c r="P1255" s="10"/>
       <c r="Q1255" s="43"/>
@@ -51367,7 +51452,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="1256" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1256" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A1256" s="7" t="s">
         <v>2</v>
       </c>
@@ -51399,8 +51484,8 @@
       <c r="L1256" s="30"/>
       <c r="M1256" s="80"/>
       <c r="N1256" s="37"/>
-      <c r="O1256" s="166">
-        <v>249</v>
+      <c r="O1256" s="218">
+        <v>255</v>
       </c>
       <c r="P1256" s="10"/>
       <c r="Q1256" s="43"/>
@@ -51440,8 +51525,8 @@
       <c r="L1257" s="30"/>
       <c r="M1257" s="80"/>
       <c r="N1257" s="37"/>
-      <c r="O1257" s="166">
-        <v>249</v>
+      <c r="O1257" s="218">
+        <v>255</v>
       </c>
       <c r="P1257" s="10"/>
       <c r="Q1257" s="43"/>
@@ -51477,7 +51562,9 @@
       <c r="L1258" s="10"/>
       <c r="M1258" s="40"/>
       <c r="N1258" s="37"/>
-      <c r="O1258" s="166"/>
+      <c r="O1258" s="218" t="s">
+        <v>339</v>
+      </c>
       <c r="P1258" s="10"/>
       <c r="Q1258" s="44" t="s">
         <v>15</v>
@@ -51514,7 +51601,7 @@
       <c r="L1259" s="10"/>
       <c r="M1259" s="40"/>
       <c r="N1259" s="37"/>
-      <c r="O1259" s="166"/>
+      <c r="O1259" s="218"/>
       <c r="P1259" s="10"/>
       <c r="Q1259" s="44" t="s">
         <v>15</v>
@@ -51551,7 +51638,7 @@
       <c r="L1260" s="10"/>
       <c r="M1260" s="40"/>
       <c r="N1260" s="37"/>
-      <c r="O1260" s="166"/>
+      <c r="O1260" s="218"/>
       <c r="P1260" s="10"/>
       <c r="Q1260" s="44" t="s">
         <v>15</v>
@@ -51588,7 +51675,9 @@
       <c r="L1261" s="10"/>
       <c r="M1261" s="40"/>
       <c r="N1261" s="37"/>
-      <c r="O1261" s="166"/>
+      <c r="O1261" s="218" t="s">
+        <v>23</v>
+      </c>
       <c r="P1261" s="10"/>
       <c r="Q1261" s="44" t="s">
         <v>15</v>
@@ -51625,7 +51714,9 @@
       <c r="L1262" s="10"/>
       <c r="M1262" s="40"/>
       <c r="N1262" s="37"/>
-      <c r="O1262" s="166"/>
+      <c r="O1262" s="218" t="s">
+        <v>335</v>
+      </c>
       <c r="P1262" s="10"/>
       <c r="Q1262" s="44" t="s">
         <v>15</v>
@@ -51662,7 +51753,9 @@
       <c r="L1263" s="10"/>
       <c r="M1263" s="40"/>
       <c r="N1263" s="37"/>
-      <c r="O1263" s="166"/>
+      <c r="O1263" s="218" t="s">
+        <v>336</v>
+      </c>
       <c r="P1263" s="10"/>
       <c r="Q1263" s="44" t="s">
         <v>15</v>
@@ -51671,7 +51764,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="1264" spans="1:18" ht="14.25" x14ac:dyDescent="0.25">
+    <row r="1264" spans="1:18" ht="15" x14ac:dyDescent="0.25">
       <c r="A1264" s="46" t="s">
         <v>2</v>
       </c>
@@ -51699,7 +51792,9 @@
       <c r="L1264" s="52"/>
       <c r="M1264" s="54"/>
       <c r="N1264" s="55"/>
-      <c r="O1264" s="167"/>
+      <c r="O1264" s="239" t="s">
+        <v>338</v>
+      </c>
       <c r="P1264" s="52"/>
       <c r="Q1264" s="57" t="s">
         <v>15</v>
@@ -51850,8 +51945,8 @@
       <c r="L1268" s="30"/>
       <c r="M1268" s="80"/>
       <c r="N1268" s="37"/>
-      <c r="O1268" s="166">
-        <v>249</v>
+      <c r="O1268" s="240">
+        <v>215</v>
       </c>
       <c r="P1268" s="10"/>
       <c r="Q1268" s="43"/>
@@ -51859,7 +51954,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="1269" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1269" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A1269" s="7" t="s">
         <v>2</v>
       </c>
@@ -51891,8 +51986,8 @@
       <c r="L1269" s="30"/>
       <c r="M1269" s="80"/>
       <c r="N1269" s="37"/>
-      <c r="O1269" s="166">
-        <v>249</v>
+      <c r="O1269" s="240">
+        <v>246</v>
       </c>
       <c r="P1269" s="10"/>
       <c r="Q1269" s="43"/>
@@ -51932,8 +52027,8 @@
       <c r="L1270" s="30"/>
       <c r="M1270" s="80"/>
       <c r="N1270" s="37"/>
-      <c r="O1270" s="166">
-        <v>249</v>
+      <c r="O1270" s="240">
+        <v>254</v>
       </c>
       <c r="P1270" s="10"/>
       <c r="Q1270" s="43"/>
@@ -51969,7 +52064,9 @@
       <c r="L1271" s="10"/>
       <c r="M1271" s="40"/>
       <c r="N1271" s="37"/>
-      <c r="O1271" s="166"/>
+      <c r="O1271" s="240" t="s">
+        <v>340</v>
+      </c>
       <c r="P1271" s="10"/>
       <c r="Q1271" s="44" t="s">
         <v>15</v>
@@ -52006,7 +52103,7 @@
       <c r="L1272" s="10"/>
       <c r="M1272" s="40"/>
       <c r="N1272" s="37"/>
-      <c r="O1272" s="166"/>
+      <c r="O1272" s="240"/>
       <c r="P1272" s="10"/>
       <c r="Q1272" s="44" t="s">
         <v>15</v>
@@ -52043,7 +52140,9 @@
       <c r="L1273" s="10"/>
       <c r="M1273" s="40"/>
       <c r="N1273" s="37"/>
-      <c r="O1273" s="166"/>
+      <c r="O1273" s="240" t="s">
+        <v>342</v>
+      </c>
       <c r="P1273" s="10"/>
       <c r="Q1273" s="44" t="s">
         <v>15</v>
@@ -52080,7 +52179,9 @@
       <c r="L1274" s="10"/>
       <c r="M1274" s="40"/>
       <c r="N1274" s="37"/>
-      <c r="O1274" s="166"/>
+      <c r="O1274" s="240" t="s">
+        <v>23</v>
+      </c>
       <c r="P1274" s="10"/>
       <c r="Q1274" s="44" t="s">
         <v>15</v>
@@ -52117,7 +52218,9 @@
       <c r="L1275" s="10"/>
       <c r="M1275" s="40"/>
       <c r="N1275" s="37"/>
-      <c r="O1275" s="166"/>
+      <c r="O1275" s="240" t="s">
+        <v>205</v>
+      </c>
       <c r="P1275" s="10"/>
       <c r="Q1275" s="44" t="s">
         <v>15</v>
@@ -52154,7 +52257,9 @@
       <c r="L1276" s="10"/>
       <c r="M1276" s="40"/>
       <c r="N1276" s="37"/>
-      <c r="O1276" s="166"/>
+      <c r="O1276" s="240" t="s">
+        <v>207</v>
+      </c>
       <c r="P1276" s="10"/>
       <c r="Q1276" s="44" t="s">
         <v>15</v>
@@ -52163,7 +52268,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="1277" spans="1:18" ht="14.25" x14ac:dyDescent="0.25">
+    <row r="1277" spans="1:18" ht="15" x14ac:dyDescent="0.25">
       <c r="A1277" s="46" t="s">
         <v>2</v>
       </c>
@@ -52191,7 +52296,9 @@
       <c r="L1277" s="52"/>
       <c r="M1277" s="54"/>
       <c r="N1277" s="55"/>
-      <c r="O1277" s="167"/>
+      <c r="O1277" s="241" t="s">
+        <v>341</v>
+      </c>
       <c r="P1277" s="52"/>
       <c r="Q1277" s="57" t="s">
         <v>15</v>
@@ -52351,7 +52458,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="1282" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1282" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
       <c r="A1282" s="7" t="s">
         <v>2</v>
       </c>
@@ -52693,87 +52800,1563 @@
       </c>
     </row>
     <row r="1291" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A1291" s="7"/>
-      <c r="B1291" s="28"/>
-      <c r="C1291" s="41"/>
-      <c r="D1291" s="30"/>
-      <c r="E1291" s="31"/>
-      <c r="F1291" s="28"/>
-      <c r="G1291" s="41"/>
-      <c r="H1291" s="30"/>
-      <c r="I1291" s="31"/>
-      <c r="J1291" s="28"/>
-      <c r="K1291" s="41"/>
-      <c r="L1291" s="30"/>
+      <c r="A1291" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1291" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1291" s="59">
+        <f>C822+1</f>
+        <v>137</v>
+      </c>
+      <c r="D1291" s="30">
+        <v>1</v>
+      </c>
+      <c r="E1291" s="31" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1291" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="G1291" s="9"/>
+      <c r="H1291" s="10"/>
+      <c r="I1291" s="7"/>
+      <c r="J1291" s="8"/>
+      <c r="K1291" s="9"/>
+      <c r="L1291" s="10"/>
       <c r="M1291" s="40"/>
-      <c r="N1291" s="220"/>
-      <c r="O1291" s="38"/>
-      <c r="P1291" s="221"/>
-      <c r="Q1291" s="43"/>
-      <c r="R1291" s="27"/>
+      <c r="N1291" s="60"/>
+      <c r="O1291" s="24">
+        <f>$C1291</f>
+        <v>137</v>
+      </c>
+      <c r="P1291" s="25"/>
+      <c r="Q1291" s="13"/>
+      <c r="R1291" s="27" t="s">
+        <v>37</v>
+      </c>
     </row>
     <row r="1292" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A1292" s="7"/>
-      <c r="B1292" s="28"/>
-      <c r="C1292" s="41"/>
-      <c r="D1292" s="30"/>
-      <c r="E1292" s="31"/>
-      <c r="F1292" s="28"/>
-      <c r="G1292" s="41"/>
-      <c r="H1292" s="30"/>
-      <c r="I1292" s="31"/>
-      <c r="J1292" s="28"/>
-      <c r="K1292" s="41"/>
-      <c r="L1292" s="30"/>
-      <c r="M1292" s="40"/>
-      <c r="N1292" s="220"/>
+      <c r="A1292" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1292" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1292" s="29">
+        <f>C1291</f>
+        <v>137</v>
+      </c>
+      <c r="D1292" s="30">
+        <v>1</v>
+      </c>
+      <c r="E1292" s="31" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1292" s="28" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1292" s="32"/>
+      <c r="H1292" s="33"/>
+      <c r="I1292" s="34"/>
+      <c r="J1292" s="35"/>
+      <c r="K1292" s="32"/>
+      <c r="L1292" s="33"/>
+      <c r="M1292" s="36"/>
+      <c r="N1292" s="37"/>
       <c r="O1292" s="38"/>
-      <c r="P1292" s="221"/>
-      <c r="Q1292" s="43"/>
-      <c r="R1292" s="27"/>
+      <c r="P1292" s="10"/>
+      <c r="Q1292" s="39"/>
+      <c r="R1292" s="27" t="s">
+        <v>5</v>
+      </c>
     </row>
     <row r="1293" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A1293" s="7"/>
-      <c r="B1293" s="28"/>
-      <c r="C1293" s="41"/>
-      <c r="D1293" s="30"/>
-      <c r="E1293" s="31"/>
-      <c r="F1293" s="28"/>
-      <c r="G1293" s="41"/>
-      <c r="H1293" s="30"/>
-      <c r="I1293" s="31"/>
-      <c r="J1293" s="28"/>
-      <c r="K1293" s="41"/>
-      <c r="L1293" s="30"/>
+      <c r="A1293" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1293" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1293" s="29">
+        <f t="shared" ref="C1293:C1303" si="99">C1292</f>
+        <v>137</v>
+      </c>
+      <c r="D1293" s="30">
+        <v>1</v>
+      </c>
+      <c r="E1293" s="31" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1293" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="G1293" s="9"/>
+      <c r="H1293" s="10"/>
+      <c r="I1293" s="7"/>
+      <c r="J1293" s="8"/>
+      <c r="K1293" s="9"/>
+      <c r="L1293" s="10"/>
       <c r="M1293" s="40"/>
-      <c r="N1293" s="220"/>
-      <c r="O1293" s="38"/>
-      <c r="P1293" s="221"/>
-      <c r="Q1293" s="43"/>
-      <c r="R1293" s="27"/>
+      <c r="N1293" s="37"/>
+      <c r="O1293" s="12">
+        <v>2</v>
+      </c>
+      <c r="P1293" s="10"/>
+      <c r="Q1293" s="13"/>
+      <c r="R1293" s="27" t="s">
+        <v>7</v>
+      </c>
     </row>
     <row r="1294" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A1294" s="7"/>
-      <c r="B1294" s="28"/>
-      <c r="C1294" s="41"/>
-      <c r="D1294" s="30"/>
-      <c r="E1294" s="31"/>
-      <c r="F1294" s="28"/>
-      <c r="G1294" s="41"/>
-      <c r="H1294" s="30"/>
+      <c r="A1294" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1294" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1294" s="29">
+        <f t="shared" si="99"/>
+        <v>137</v>
+      </c>
+      <c r="D1294" s="30">
+        <v>1</v>
+      </c>
+      <c r="E1294" s="31" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1294" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="G1294" s="41">
+        <v>1</v>
+      </c>
+      <c r="H1294" s="30">
+        <v>1</v>
+      </c>
       <c r="I1294" s="31"/>
       <c r="J1294" s="28"/>
       <c r="K1294" s="41"/>
       <c r="L1294" s="30"/>
-      <c r="M1294" s="40"/>
-      <c r="N1294" s="220"/>
-      <c r="O1294" s="38"/>
-      <c r="P1294" s="221"/>
+      <c r="M1294" s="80"/>
+      <c r="N1294" s="37"/>
+      <c r="O1294" s="166">
+        <v>249</v>
+      </c>
+      <c r="P1294" s="10"/>
       <c r="Q1294" s="43"/>
-      <c r="R1294" s="27"/>
-    </row>
-    <row r="1295" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A1295" s="222"/>
+      <c r="R1294" s="27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1295" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A1295" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1295" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1295" s="29">
+        <f t="shared" si="99"/>
+        <v>137</v>
+      </c>
+      <c r="D1295" s="30">
+        <v>1</v>
+      </c>
+      <c r="E1295" s="31" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1295" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="G1295" s="41">
+        <v>1</v>
+      </c>
+      <c r="H1295" s="30">
+        <v>2</v>
+      </c>
+      <c r="I1295" s="31"/>
+      <c r="J1295" s="28"/>
+      <c r="K1295" s="41"/>
+      <c r="L1295" s="30"/>
+      <c r="M1295" s="80"/>
+      <c r="N1295" s="37"/>
+      <c r="O1295" s="166">
+        <v>249</v>
+      </c>
+      <c r="P1295" s="10"/>
+      <c r="Q1295" s="43"/>
+      <c r="R1295" s="27" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="1296" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1296" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1296" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1296" s="29">
+        <f t="shared" si="99"/>
+        <v>137</v>
+      </c>
+      <c r="D1296" s="30">
+        <v>1</v>
+      </c>
+      <c r="E1296" s="31" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1296" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="G1296" s="41">
+        <v>1</v>
+      </c>
+      <c r="H1296" s="30">
+        <v>3</v>
+      </c>
+      <c r="I1296" s="31"/>
+      <c r="J1296" s="28"/>
+      <c r="K1296" s="41"/>
+      <c r="L1296" s="30"/>
+      <c r="M1296" s="80"/>
+      <c r="N1296" s="37"/>
+      <c r="O1296" s="166">
+        <v>249</v>
+      </c>
+      <c r="P1296" s="10"/>
+      <c r="Q1296" s="43"/>
+      <c r="R1296" s="27" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1297" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1297" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1297" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1297" s="29">
+        <f t="shared" si="99"/>
+        <v>137</v>
+      </c>
+      <c r="D1297" s="30">
+        <v>1</v>
+      </c>
+      <c r="E1297" s="31" t="s">
+        <v>12</v>
+      </c>
+      <c r="F1297" s="28" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1297" s="9"/>
+      <c r="H1297" s="10"/>
+      <c r="I1297" s="7"/>
+      <c r="J1297" s="8"/>
+      <c r="K1297" s="9"/>
+      <c r="L1297" s="10"/>
+      <c r="M1297" s="40"/>
+      <c r="N1297" s="37"/>
+      <c r="O1297" s="166"/>
+      <c r="P1297" s="10"/>
+      <c r="Q1297" s="44" t="s">
+        <v>15</v>
+      </c>
+      <c r="R1297" s="45" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="1298" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1298" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1298" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1298" s="29">
+        <f t="shared" si="99"/>
+        <v>137</v>
+      </c>
+      <c r="D1298" s="30">
+        <v>1</v>
+      </c>
+      <c r="E1298" s="31" t="s">
+        <v>17</v>
+      </c>
+      <c r="F1298" s="28" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1298" s="9"/>
+      <c r="H1298" s="10"/>
+      <c r="I1298" s="7"/>
+      <c r="J1298" s="8"/>
+      <c r="K1298" s="9"/>
+      <c r="L1298" s="10"/>
+      <c r="M1298" s="40"/>
+      <c r="N1298" s="37"/>
+      <c r="O1298" s="166"/>
+      <c r="P1298" s="10"/>
+      <c r="Q1298" s="44" t="s">
+        <v>15</v>
+      </c>
+      <c r="R1298" s="45" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="1299" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1299" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1299" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1299" s="29">
+        <f t="shared" si="99"/>
+        <v>137</v>
+      </c>
+      <c r="D1299" s="30">
+        <v>1</v>
+      </c>
+      <c r="E1299" s="31" t="s">
+        <v>19</v>
+      </c>
+      <c r="F1299" s="28" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1299" s="9"/>
+      <c r="H1299" s="10"/>
+      <c r="I1299" s="7"/>
+      <c r="J1299" s="8"/>
+      <c r="K1299" s="9"/>
+      <c r="L1299" s="10"/>
+      <c r="M1299" s="40"/>
+      <c r="N1299" s="37"/>
+      <c r="O1299" s="166"/>
+      <c r="P1299" s="10"/>
+      <c r="Q1299" s="44" t="s">
+        <v>15</v>
+      </c>
+      <c r="R1299" s="45" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="1300" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1300" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1300" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1300" s="29">
+        <f t="shared" si="99"/>
+        <v>137</v>
+      </c>
+      <c r="D1300" s="30">
+        <v>1</v>
+      </c>
+      <c r="E1300" s="31" t="s">
+        <v>22</v>
+      </c>
+      <c r="F1300" s="28" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1300" s="9"/>
+      <c r="H1300" s="10"/>
+      <c r="I1300" s="7"/>
+      <c r="J1300" s="8"/>
+      <c r="K1300" s="9"/>
+      <c r="L1300" s="10"/>
+      <c r="M1300" s="40"/>
+      <c r="N1300" s="37"/>
+      <c r="O1300" s="166"/>
+      <c r="P1300" s="10"/>
+      <c r="Q1300" s="44" t="s">
+        <v>15</v>
+      </c>
+      <c r="R1300" s="45" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="1301" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1301" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1301" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1301" s="29">
+        <f t="shared" si="99"/>
+        <v>137</v>
+      </c>
+      <c r="D1301" s="30">
+        <v>1</v>
+      </c>
+      <c r="E1301" s="31" t="s">
+        <v>25</v>
+      </c>
+      <c r="F1301" s="28" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1301" s="9"/>
+      <c r="H1301" s="10"/>
+      <c r="I1301" s="7"/>
+      <c r="J1301" s="8"/>
+      <c r="K1301" s="9"/>
+      <c r="L1301" s="10"/>
+      <c r="M1301" s="40"/>
+      <c r="N1301" s="37"/>
+      <c r="O1301" s="166"/>
+      <c r="P1301" s="10"/>
+      <c r="Q1301" s="44" t="s">
+        <v>15</v>
+      </c>
+      <c r="R1301" s="27" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="1302" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1302" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1302" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1302" s="29">
+        <f t="shared" si="99"/>
+        <v>137</v>
+      </c>
+      <c r="D1302" s="30">
+        <v>1</v>
+      </c>
+      <c r="E1302" s="31" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1302" s="28" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1302" s="9"/>
+      <c r="H1302" s="10"/>
+      <c r="I1302" s="7"/>
+      <c r="J1302" s="8"/>
+      <c r="K1302" s="9"/>
+      <c r="L1302" s="10"/>
+      <c r="M1302" s="40"/>
+      <c r="N1302" s="37"/>
+      <c r="O1302" s="166"/>
+      <c r="P1302" s="10"/>
+      <c r="Q1302" s="44" t="s">
+        <v>15</v>
+      </c>
+      <c r="R1302" s="27" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="1303" spans="1:18" ht="14.25" x14ac:dyDescent="0.25">
+      <c r="A1303" s="46" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1303" s="47" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1303" s="48">
+        <f t="shared" si="99"/>
+        <v>137</v>
+      </c>
+      <c r="D1303" s="49">
+        <v>1</v>
+      </c>
+      <c r="E1303" s="50" t="s">
+        <v>33</v>
+      </c>
+      <c r="F1303" s="47" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1303" s="51"/>
+      <c r="H1303" s="52"/>
+      <c r="I1303" s="46"/>
+      <c r="J1303" s="53"/>
+      <c r="K1303" s="51"/>
+      <c r="L1303" s="52"/>
+      <c r="M1303" s="54"/>
+      <c r="N1303" s="55"/>
+      <c r="O1303" s="167"/>
+      <c r="P1303" s="52"/>
+      <c r="Q1303" s="57" t="s">
+        <v>15</v>
+      </c>
+      <c r="R1303" s="58" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="1304" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1304" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1304" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1304" s="59">
+        <f>C835+1</f>
+        <v>138</v>
+      </c>
+      <c r="D1304" s="30">
+        <v>1</v>
+      </c>
+      <c r="E1304" s="31" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1304" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="G1304" s="9"/>
+      <c r="H1304" s="10"/>
+      <c r="I1304" s="7"/>
+      <c r="J1304" s="8"/>
+      <c r="K1304" s="9"/>
+      <c r="L1304" s="10"/>
+      <c r="M1304" s="40"/>
+      <c r="N1304" s="60"/>
+      <c r="O1304" s="24">
+        <f>$C1304</f>
+        <v>138</v>
+      </c>
+      <c r="P1304" s="25"/>
+      <c r="Q1304" s="13"/>
+      <c r="R1304" s="27" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="1305" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1305" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1305" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1305" s="29">
+        <f>C1304</f>
+        <v>138</v>
+      </c>
+      <c r="D1305" s="30">
+        <v>1</v>
+      </c>
+      <c r="E1305" s="31" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1305" s="28" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1305" s="32"/>
+      <c r="H1305" s="33"/>
+      <c r="I1305" s="34"/>
+      <c r="J1305" s="35"/>
+      <c r="K1305" s="32"/>
+      <c r="L1305" s="33"/>
+      <c r="M1305" s="36"/>
+      <c r="N1305" s="37"/>
+      <c r="O1305" s="38"/>
+      <c r="P1305" s="10"/>
+      <c r="Q1305" s="39"/>
+      <c r="R1305" s="27" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1306" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1306" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1306" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1306" s="29">
+        <f t="shared" ref="C1306:C1316" si="100">C1305</f>
+        <v>138</v>
+      </c>
+      <c r="D1306" s="30">
+        <v>1</v>
+      </c>
+      <c r="E1306" s="31" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1306" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="G1306" s="9"/>
+      <c r="H1306" s="10"/>
+      <c r="I1306" s="7"/>
+      <c r="J1306" s="8"/>
+      <c r="K1306" s="9"/>
+      <c r="L1306" s="10"/>
+      <c r="M1306" s="40"/>
+      <c r="N1306" s="37"/>
+      <c r="O1306" s="12">
+        <v>2</v>
+      </c>
+      <c r="P1306" s="10"/>
+      <c r="Q1306" s="13"/>
+      <c r="R1306" s="27" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="1307" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1307" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1307" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1307" s="29">
+        <f t="shared" si="100"/>
+        <v>138</v>
+      </c>
+      <c r="D1307" s="30">
+        <v>1</v>
+      </c>
+      <c r="E1307" s="31" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1307" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="G1307" s="41">
+        <v>1</v>
+      </c>
+      <c r="H1307" s="30">
+        <v>1</v>
+      </c>
+      <c r="I1307" s="31"/>
+      <c r="J1307" s="28"/>
+      <c r="K1307" s="41"/>
+      <c r="L1307" s="30"/>
+      <c r="M1307" s="80"/>
+      <c r="N1307" s="37"/>
+      <c r="O1307" s="166">
+        <v>249</v>
+      </c>
+      <c r="P1307" s="10"/>
+      <c r="Q1307" s="43"/>
+      <c r="R1307" s="27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1308" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A1308" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1308" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1308" s="29">
+        <f t="shared" si="100"/>
+        <v>138</v>
+      </c>
+      <c r="D1308" s="30">
+        <v>1</v>
+      </c>
+      <c r="E1308" s="31" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1308" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="G1308" s="41">
+        <v>1</v>
+      </c>
+      <c r="H1308" s="30">
+        <v>2</v>
+      </c>
+      <c r="I1308" s="31"/>
+      <c r="J1308" s="28"/>
+      <c r="K1308" s="41"/>
+      <c r="L1308" s="30"/>
+      <c r="M1308" s="80"/>
+      <c r="N1308" s="37"/>
+      <c r="O1308" s="166">
+        <v>249</v>
+      </c>
+      <c r="P1308" s="10"/>
+      <c r="Q1308" s="43"/>
+      <c r="R1308" s="27" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="1309" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1309" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1309" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1309" s="29">
+        <f t="shared" si="100"/>
+        <v>138</v>
+      </c>
+      <c r="D1309" s="30">
+        <v>1</v>
+      </c>
+      <c r="E1309" s="31" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1309" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="G1309" s="41">
+        <v>1</v>
+      </c>
+      <c r="H1309" s="30">
+        <v>3</v>
+      </c>
+      <c r="I1309" s="31"/>
+      <c r="J1309" s="28"/>
+      <c r="K1309" s="41"/>
+      <c r="L1309" s="30"/>
+      <c r="M1309" s="80"/>
+      <c r="N1309" s="37"/>
+      <c r="O1309" s="166">
+        <v>249</v>
+      </c>
+      <c r="P1309" s="10"/>
+      <c r="Q1309" s="43"/>
+      <c r="R1309" s="27" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1310" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1310" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1310" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1310" s="29">
+        <f t="shared" si="100"/>
+        <v>138</v>
+      </c>
+      <c r="D1310" s="30">
+        <v>1</v>
+      </c>
+      <c r="E1310" s="31" t="s">
+        <v>12</v>
+      </c>
+      <c r="F1310" s="28" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1310" s="9"/>
+      <c r="H1310" s="10"/>
+      <c r="I1310" s="7"/>
+      <c r="J1310" s="8"/>
+      <c r="K1310" s="9"/>
+      <c r="L1310" s="10"/>
+      <c r="M1310" s="40"/>
+      <c r="N1310" s="37"/>
+      <c r="O1310" s="166"/>
+      <c r="P1310" s="10"/>
+      <c r="Q1310" s="44" t="s">
+        <v>15</v>
+      </c>
+      <c r="R1310" s="45" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="1311" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1311" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1311" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1311" s="29">
+        <f t="shared" si="100"/>
+        <v>138</v>
+      </c>
+      <c r="D1311" s="30">
+        <v>1</v>
+      </c>
+      <c r="E1311" s="31" t="s">
+        <v>17</v>
+      </c>
+      <c r="F1311" s="28" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1311" s="9"/>
+      <c r="H1311" s="10"/>
+      <c r="I1311" s="7"/>
+      <c r="J1311" s="8"/>
+      <c r="K1311" s="9"/>
+      <c r="L1311" s="10"/>
+      <c r="M1311" s="40"/>
+      <c r="N1311" s="37"/>
+      <c r="O1311" s="166"/>
+      <c r="P1311" s="10"/>
+      <c r="Q1311" s="44" t="s">
+        <v>15</v>
+      </c>
+      <c r="R1311" s="45" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="1312" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1312" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1312" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1312" s="29">
+        <f t="shared" si="100"/>
+        <v>138</v>
+      </c>
+      <c r="D1312" s="30">
+        <v>1</v>
+      </c>
+      <c r="E1312" s="31" t="s">
+        <v>19</v>
+      </c>
+      <c r="F1312" s="28" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1312" s="9"/>
+      <c r="H1312" s="10"/>
+      <c r="I1312" s="7"/>
+      <c r="J1312" s="8"/>
+      <c r="K1312" s="9"/>
+      <c r="L1312" s="10"/>
+      <c r="M1312" s="40"/>
+      <c r="N1312" s="37"/>
+      <c r="O1312" s="166"/>
+      <c r="P1312" s="10"/>
+      <c r="Q1312" s="44" t="s">
+        <v>15</v>
+      </c>
+      <c r="R1312" s="45" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="1313" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1313" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1313" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1313" s="29">
+        <f t="shared" si="100"/>
+        <v>138</v>
+      </c>
+      <c r="D1313" s="30">
+        <v>1</v>
+      </c>
+      <c r="E1313" s="31" t="s">
+        <v>22</v>
+      </c>
+      <c r="F1313" s="28" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1313" s="9"/>
+      <c r="H1313" s="10"/>
+      <c r="I1313" s="7"/>
+      <c r="J1313" s="8"/>
+      <c r="K1313" s="9"/>
+      <c r="L1313" s="10"/>
+      <c r="M1313" s="40"/>
+      <c r="N1313" s="37"/>
+      <c r="O1313" s="166"/>
+      <c r="P1313" s="10"/>
+      <c r="Q1313" s="44" t="s">
+        <v>15</v>
+      </c>
+      <c r="R1313" s="45" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="1314" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1314" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1314" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1314" s="29">
+        <f t="shared" si="100"/>
+        <v>138</v>
+      </c>
+      <c r="D1314" s="30">
+        <v>1</v>
+      </c>
+      <c r="E1314" s="31" t="s">
+        <v>25</v>
+      </c>
+      <c r="F1314" s="28" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1314" s="9"/>
+      <c r="H1314" s="10"/>
+      <c r="I1314" s="7"/>
+      <c r="J1314" s="8"/>
+      <c r="K1314" s="9"/>
+      <c r="L1314" s="10"/>
+      <c r="M1314" s="40"/>
+      <c r="N1314" s="37"/>
+      <c r="O1314" s="166"/>
+      <c r="P1314" s="10"/>
+      <c r="Q1314" s="44" t="s">
+        <v>15</v>
+      </c>
+      <c r="R1314" s="27" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="1315" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1315" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1315" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1315" s="29">
+        <f t="shared" si="100"/>
+        <v>138</v>
+      </c>
+      <c r="D1315" s="30">
+        <v>1</v>
+      </c>
+      <c r="E1315" s="31" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1315" s="28" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1315" s="9"/>
+      <c r="H1315" s="10"/>
+      <c r="I1315" s="7"/>
+      <c r="J1315" s="8"/>
+      <c r="K1315" s="9"/>
+      <c r="L1315" s="10"/>
+      <c r="M1315" s="40"/>
+      <c r="N1315" s="37"/>
+      <c r="O1315" s="166"/>
+      <c r="P1315" s="10"/>
+      <c r="Q1315" s="44" t="s">
+        <v>15</v>
+      </c>
+      <c r="R1315" s="27" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="1316" spans="1:18" ht="14.25" x14ac:dyDescent="0.25">
+      <c r="A1316" s="46" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1316" s="47" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1316" s="48">
+        <f t="shared" si="100"/>
+        <v>138</v>
+      </c>
+      <c r="D1316" s="49">
+        <v>1</v>
+      </c>
+      <c r="E1316" s="50" t="s">
+        <v>33</v>
+      </c>
+      <c r="F1316" s="47" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1316" s="51"/>
+      <c r="H1316" s="52"/>
+      <c r="I1316" s="46"/>
+      <c r="J1316" s="53"/>
+      <c r="K1316" s="51"/>
+      <c r="L1316" s="52"/>
+      <c r="M1316" s="54"/>
+      <c r="N1316" s="55"/>
+      <c r="O1316" s="167"/>
+      <c r="P1316" s="52"/>
+      <c r="Q1316" s="57" t="s">
+        <v>15</v>
+      </c>
+      <c r="R1316" s="58" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="1317" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1317" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1317" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1317" s="59">
+        <f>C848+1</f>
+        <v>139</v>
+      </c>
+      <c r="D1317" s="30">
+        <v>1</v>
+      </c>
+      <c r="E1317" s="31" t="s">
+        <v>3</v>
+      </c>
+      <c r="F1317" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="G1317" s="9"/>
+      <c r="H1317" s="10"/>
+      <c r="I1317" s="7"/>
+      <c r="J1317" s="8"/>
+      <c r="K1317" s="9"/>
+      <c r="L1317" s="10"/>
+      <c r="M1317" s="40"/>
+      <c r="N1317" s="60"/>
+      <c r="O1317" s="24">
+        <f>$C1317</f>
+        <v>139</v>
+      </c>
+      <c r="P1317" s="25"/>
+      <c r="Q1317" s="13"/>
+      <c r="R1317" s="27" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="1318" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1318" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1318" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1318" s="29">
+        <f>C1317</f>
+        <v>139</v>
+      </c>
+      <c r="D1318" s="30">
+        <v>1</v>
+      </c>
+      <c r="E1318" s="31" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1318" s="28" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1318" s="32"/>
+      <c r="H1318" s="33"/>
+      <c r="I1318" s="34"/>
+      <c r="J1318" s="35"/>
+      <c r="K1318" s="32"/>
+      <c r="L1318" s="33"/>
+      <c r="M1318" s="36"/>
+      <c r="N1318" s="37"/>
+      <c r="O1318" s="38"/>
+      <c r="P1318" s="10"/>
+      <c r="Q1318" s="39"/>
+      <c r="R1318" s="27" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="1319" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1319" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1319" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1319" s="29">
+        <f t="shared" ref="C1319:C1329" si="101">C1318</f>
+        <v>139</v>
+      </c>
+      <c r="D1319" s="30">
+        <v>1</v>
+      </c>
+      <c r="E1319" s="31" t="s">
+        <v>6</v>
+      </c>
+      <c r="F1319" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="G1319" s="9"/>
+      <c r="H1319" s="10"/>
+      <c r="I1319" s="7"/>
+      <c r="J1319" s="8"/>
+      <c r="K1319" s="9"/>
+      <c r="L1319" s="10"/>
+      <c r="M1319" s="40"/>
+      <c r="N1319" s="37"/>
+      <c r="O1319" s="12">
+        <v>2</v>
+      </c>
+      <c r="P1319" s="10"/>
+      <c r="Q1319" s="13"/>
+      <c r="R1319" s="27" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="1320" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1320" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1320" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1320" s="29">
+        <f t="shared" si="101"/>
+        <v>139</v>
+      </c>
+      <c r="D1320" s="30">
+        <v>1</v>
+      </c>
+      <c r="E1320" s="31" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1320" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="G1320" s="41">
+        <v>1</v>
+      </c>
+      <c r="H1320" s="30">
+        <v>1</v>
+      </c>
+      <c r="I1320" s="31"/>
+      <c r="J1320" s="28"/>
+      <c r="K1320" s="41"/>
+      <c r="L1320" s="30"/>
+      <c r="M1320" s="80"/>
+      <c r="N1320" s="37"/>
+      <c r="O1320" s="166">
+        <v>249</v>
+      </c>
+      <c r="P1320" s="10"/>
+      <c r="Q1320" s="43"/>
+      <c r="R1320" s="27" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="1321" spans="1:18" ht="25.5" x14ac:dyDescent="0.25">
+      <c r="A1321" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1321" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1321" s="29">
+        <f t="shared" si="101"/>
+        <v>139</v>
+      </c>
+      <c r="D1321" s="30">
+        <v>1</v>
+      </c>
+      <c r="E1321" s="31" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1321" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="G1321" s="41">
+        <v>1</v>
+      </c>
+      <c r="H1321" s="30">
+        <v>2</v>
+      </c>
+      <c r="I1321" s="31"/>
+      <c r="J1321" s="28"/>
+      <c r="K1321" s="41"/>
+      <c r="L1321" s="30"/>
+      <c r="M1321" s="80"/>
+      <c r="N1321" s="37"/>
+      <c r="O1321" s="166">
+        <v>249</v>
+      </c>
+      <c r="P1321" s="10"/>
+      <c r="Q1321" s="43"/>
+      <c r="R1321" s="27" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="1322" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1322" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1322" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1322" s="29">
+        <f t="shared" si="101"/>
+        <v>139</v>
+      </c>
+      <c r="D1322" s="30">
+        <v>1</v>
+      </c>
+      <c r="E1322" s="31" t="s">
+        <v>8</v>
+      </c>
+      <c r="F1322" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="G1322" s="41">
+        <v>1</v>
+      </c>
+      <c r="H1322" s="30">
+        <v>3</v>
+      </c>
+      <c r="I1322" s="31"/>
+      <c r="J1322" s="28"/>
+      <c r="K1322" s="41"/>
+      <c r="L1322" s="30"/>
+      <c r="M1322" s="80"/>
+      <c r="N1322" s="37"/>
+      <c r="O1322" s="166">
+        <v>249</v>
+      </c>
+      <c r="P1322" s="10"/>
+      <c r="Q1322" s="43"/>
+      <c r="R1322" s="27" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="1323" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1323" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1323" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1323" s="29">
+        <f t="shared" si="101"/>
+        <v>139</v>
+      </c>
+      <c r="D1323" s="30">
+        <v>1</v>
+      </c>
+      <c r="E1323" s="31" t="s">
+        <v>12</v>
+      </c>
+      <c r="F1323" s="28" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1323" s="9"/>
+      <c r="H1323" s="10"/>
+      <c r="I1323" s="7"/>
+      <c r="J1323" s="8"/>
+      <c r="K1323" s="9"/>
+      <c r="L1323" s="10"/>
+      <c r="M1323" s="40"/>
+      <c r="N1323" s="37"/>
+      <c r="O1323" s="166"/>
+      <c r="P1323" s="10"/>
+      <c r="Q1323" s="44" t="s">
+        <v>15</v>
+      </c>
+      <c r="R1323" s="45" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="1324" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1324" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1324" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1324" s="29">
+        <f t="shared" si="101"/>
+        <v>139</v>
+      </c>
+      <c r="D1324" s="30">
+        <v>1</v>
+      </c>
+      <c r="E1324" s="31" t="s">
+        <v>17</v>
+      </c>
+      <c r="F1324" s="28" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1324" s="9"/>
+      <c r="H1324" s="10"/>
+      <c r="I1324" s="7"/>
+      <c r="J1324" s="8"/>
+      <c r="K1324" s="9"/>
+      <c r="L1324" s="10"/>
+      <c r="M1324" s="40"/>
+      <c r="N1324" s="37"/>
+      <c r="O1324" s="166"/>
+      <c r="P1324" s="10"/>
+      <c r="Q1324" s="44" t="s">
+        <v>15</v>
+      </c>
+      <c r="R1324" s="45" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="1325" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1325" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1325" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1325" s="29">
+        <f t="shared" si="101"/>
+        <v>139</v>
+      </c>
+      <c r="D1325" s="30">
+        <v>1</v>
+      </c>
+      <c r="E1325" s="31" t="s">
+        <v>19</v>
+      </c>
+      <c r="F1325" s="28" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1325" s="9"/>
+      <c r="H1325" s="10"/>
+      <c r="I1325" s="7"/>
+      <c r="J1325" s="8"/>
+      <c r="K1325" s="9"/>
+      <c r="L1325" s="10"/>
+      <c r="M1325" s="40"/>
+      <c r="N1325" s="37"/>
+      <c r="O1325" s="166"/>
+      <c r="P1325" s="10"/>
+      <c r="Q1325" s="44" t="s">
+        <v>15</v>
+      </c>
+      <c r="R1325" s="45" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="1326" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1326" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1326" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1326" s="29">
+        <f t="shared" si="101"/>
+        <v>139</v>
+      </c>
+      <c r="D1326" s="30">
+        <v>1</v>
+      </c>
+      <c r="E1326" s="31" t="s">
+        <v>22</v>
+      </c>
+      <c r="F1326" s="28" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1326" s="9"/>
+      <c r="H1326" s="10"/>
+      <c r="I1326" s="7"/>
+      <c r="J1326" s="8"/>
+      <c r="K1326" s="9"/>
+      <c r="L1326" s="10"/>
+      <c r="M1326" s="40"/>
+      <c r="N1326" s="37"/>
+      <c r="O1326" s="166"/>
+      <c r="P1326" s="10"/>
+      <c r="Q1326" s="44" t="s">
+        <v>15</v>
+      </c>
+      <c r="R1326" s="45" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="1327" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1327" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1327" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1327" s="29">
+        <f t="shared" si="101"/>
+        <v>139</v>
+      </c>
+      <c r="D1327" s="30">
+        <v>1</v>
+      </c>
+      <c r="E1327" s="31" t="s">
+        <v>25</v>
+      </c>
+      <c r="F1327" s="28" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1327" s="9"/>
+      <c r="H1327" s="10"/>
+      <c r="I1327" s="7"/>
+      <c r="J1327" s="8"/>
+      <c r="K1327" s="9"/>
+      <c r="L1327" s="10"/>
+      <c r="M1327" s="40"/>
+      <c r="N1327" s="37"/>
+      <c r="O1327" s="166"/>
+      <c r="P1327" s="10"/>
+      <c r="Q1327" s="44" t="s">
+        <v>15</v>
+      </c>
+      <c r="R1327" s="27" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="1328" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1328" s="7" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1328" s="28" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1328" s="29">
+        <f t="shared" si="101"/>
+        <v>139</v>
+      </c>
+      <c r="D1328" s="30">
+        <v>1</v>
+      </c>
+      <c r="E1328" s="31" t="s">
+        <v>30</v>
+      </c>
+      <c r="F1328" s="28" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1328" s="9"/>
+      <c r="H1328" s="10"/>
+      <c r="I1328" s="7"/>
+      <c r="J1328" s="8"/>
+      <c r="K1328" s="9"/>
+      <c r="L1328" s="10"/>
+      <c r="M1328" s="40"/>
+      <c r="N1328" s="37"/>
+      <c r="O1328" s="166"/>
+      <c r="P1328" s="10"/>
+      <c r="Q1328" s="44" t="s">
+        <v>15</v>
+      </c>
+      <c r="R1328" s="27" t="s">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="1329" spans="1:18" ht="14.25" x14ac:dyDescent="0.25">
+      <c r="A1329" s="46" t="s">
+        <v>2</v>
+      </c>
+      <c r="B1329" s="47" t="s">
+        <v>0</v>
+      </c>
+      <c r="C1329" s="48">
+        <f t="shared" si="101"/>
+        <v>139</v>
+      </c>
+      <c r="D1329" s="49">
+        <v>1</v>
+      </c>
+      <c r="E1329" s="50" t="s">
+        <v>33</v>
+      </c>
+      <c r="F1329" s="47" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1329" s="51"/>
+      <c r="H1329" s="52"/>
+      <c r="I1329" s="46"/>
+      <c r="J1329" s="53"/>
+      <c r="K1329" s="51"/>
+      <c r="L1329" s="52"/>
+      <c r="M1329" s="54"/>
+      <c r="N1329" s="55"/>
+      <c r="O1329" s="167"/>
+      <c r="P1329" s="52"/>
+      <c r="Q1329" s="57" t="s">
+        <v>15</v>
+      </c>
+      <c r="R1329" s="58" t="s">
+        <v>36</v>
+      </c>
+    </row>
+    <row r="1330" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1330" s="7"/>
+      <c r="B1330" s="28"/>
+      <c r="C1330" s="41"/>
+      <c r="D1330" s="30"/>
+      <c r="E1330" s="31"/>
+      <c r="F1330" s="28"/>
+      <c r="G1330" s="41"/>
+      <c r="H1330" s="30"/>
+      <c r="I1330" s="31"/>
+      <c r="J1330" s="28"/>
+      <c r="K1330" s="41"/>
+      <c r="L1330" s="30"/>
+      <c r="M1330" s="40"/>
+      <c r="N1330" s="220"/>
+      <c r="O1330" s="38"/>
+      <c r="P1330" s="221"/>
+      <c r="Q1330" s="43"/>
+      <c r="R1330" s="27"/>
+    </row>
+    <row r="1331" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1331" s="7"/>
+      <c r="B1331" s="28"/>
+      <c r="C1331" s="41"/>
+      <c r="D1331" s="30"/>
+      <c r="E1331" s="31"/>
+      <c r="F1331" s="28"/>
+      <c r="G1331" s="41"/>
+      <c r="H1331" s="30"/>
+      <c r="I1331" s="31"/>
+      <c r="J1331" s="28"/>
+      <c r="K1331" s="41"/>
+      <c r="L1331" s="30"/>
+      <c r="M1331" s="40"/>
+      <c r="N1331" s="220"/>
+      <c r="O1331" s="38"/>
+      <c r="P1331" s="221"/>
+      <c r="Q1331" s="43"/>
+      <c r="R1331" s="27"/>
+    </row>
+    <row r="1332" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1332" s="7"/>
+      <c r="B1332" s="28"/>
+      <c r="C1332" s="41"/>
+      <c r="D1332" s="30"/>
+      <c r="E1332" s="31"/>
+      <c r="F1332" s="28"/>
+      <c r="G1332" s="41"/>
+      <c r="H1332" s="30"/>
+      <c r="I1332" s="31"/>
+      <c r="J1332" s="28"/>
+      <c r="K1332" s="41"/>
+      <c r="L1332" s="30"/>
+      <c r="M1332" s="40"/>
+      <c r="N1332" s="220"/>
+      <c r="O1332" s="38"/>
+      <c r="P1332" s="221"/>
+      <c r="Q1332" s="43"/>
+      <c r="R1332" s="27"/>
+    </row>
+    <row r="1333" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1333" s="7"/>
+      <c r="B1333" s="28"/>
+      <c r="C1333" s="41"/>
+      <c r="D1333" s="30"/>
+      <c r="E1333" s="31"/>
+      <c r="F1333" s="28"/>
+      <c r="G1333" s="41"/>
+      <c r="H1333" s="30"/>
+      <c r="I1333" s="31"/>
+      <c r="J1333" s="28"/>
+      <c r="K1333" s="41"/>
+      <c r="L1333" s="30"/>
+      <c r="M1333" s="40"/>
+      <c r="N1333" s="220"/>
+      <c r="O1333" s="38"/>
+      <c r="P1333" s="221"/>
+      <c r="Q1333" s="43"/>
+      <c r="R1333" s="27"/>
+    </row>
+    <row r="1334" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A1334" s="222"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -52868,8 +54451,12 @@
     <hyperlink ref="O1199" r:id="rId84" xr:uid="{00000000-0004-0000-0000-000053000000}"/>
     <hyperlink ref="O1212" r:id="rId85" xr:uid="{4C2D4A00-3B48-410F-8B9C-1A20F07ADA41}"/>
     <hyperlink ref="O1225" r:id="rId86" xr:uid="{DD867BA2-3AC6-4F0F-8F83-4A366A7283B1}"/>
+    <hyperlink ref="O1238" r:id="rId87" xr:uid="{73D7205C-0B50-4044-AD05-79B62B974E2D}"/>
+    <hyperlink ref="O1251" r:id="rId88" xr:uid="{71FC9FF7-C407-4E65-9A4F-D76B8F53D17D}"/>
+    <hyperlink ref="O1264" r:id="rId89" xr:uid="{F08D733A-2C85-4236-B171-C4472FEAAFC4}"/>
+    <hyperlink ref="O1277" r:id="rId90" xr:uid="{33E5130C-430C-4092-8791-AF387E27A53D}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId87"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId91"/>
 </worksheet>
 </file>
</xml_diff>